<commit_message>
Fill in ONSITE prices and totals for Ustyurt GCC commercial proposal
Prices from the user's edited KP draft; line amounts and grand total
computed in both the KP letter and the RFQ form. Items 13 and 15 are
quoted as minimum ("от") prices.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019mmT6m1RtMJfg2hsA8Js6E
</commit_message>
<xml_diff>
--- a/KP/ONSITE_Ustyurt_GCC/RFQ_Chemicals_ONSITE.xlsx
+++ b/KP/ONSITE_Ustyurt_GCC/RFQ_Chemicals_ONSITE.xlsx
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="320">
   <si>
     <t xml:space="preserve">ЗАПРОС ЦЕНОВОГО ПРЕДЛОЖЕНИЯ — химические реагенты для водоподготовки, Устюртский ГХК</t>
   </si>
@@ -691,6 +691,9 @@
   <si>
     <t xml:space="preserve">услуга
 lot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цена указана «от»; окончательная стоимость уточняется / Price stated as minimum, to be confirmed</t>
   </si>
   <si>
     <t xml:space="preserve">14</t>
@@ -2281,10 +2284,12 @@
         <f aca="false">J20</f>
         <v>24500</v>
       </c>
-      <c r="O20" s="26"/>
+      <c r="O20" s="26" t="n">
+        <v>13800</v>
+      </c>
       <c r="P20" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N20),ISNUMBER(O20)),N20*O20,0)</f>
-        <v>0</v>
+        <v>338100000</v>
       </c>
       <c r="Q20" s="24" t="s">
         <v>73</v>
@@ -2337,10 +2342,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I6</f>
         <v>1800</v>
       </c>
-      <c r="O21" s="26"/>
+      <c r="O21" s="26" t="n">
+        <v>28000</v>
+      </c>
       <c r="P21" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N21),ISNUMBER(O21)),N21*O21,0)</f>
-        <v>0</v>
+        <v>50400000</v>
       </c>
       <c r="Q21" s="24" t="s">
         <v>73</v>
@@ -2393,10 +2400,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I7</f>
         <v>1800</v>
       </c>
-      <c r="O22" s="26"/>
+      <c r="O22" s="26" t="n">
+        <v>41500</v>
+      </c>
       <c r="P22" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N22),ISNUMBER(O22)),N22*O22,0)</f>
-        <v>0</v>
+        <v>74700000</v>
       </c>
       <c r="Q22" s="24" t="s">
         <v>73</v>
@@ -2450,10 +2459,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I8</f>
         <v>6440</v>
       </c>
-      <c r="O23" s="26"/>
+      <c r="O23" s="26" t="n">
+        <v>38000</v>
+      </c>
       <c r="P23" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N23),ISNUMBER(O23)),N23*O23,0)</f>
-        <v>0</v>
+        <v>244720000</v>
       </c>
       <c r="Q23" s="24" t="s">
         <v>73</v>
@@ -2531,10 +2542,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I9</f>
         <v>23000</v>
       </c>
-      <c r="O25" s="26"/>
+      <c r="O25" s="26" t="n">
+        <v>40000</v>
+      </c>
       <c r="P25" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N25),ISNUMBER(O25)),N25*O25,0)</f>
-        <v>0</v>
+        <v>920000000</v>
       </c>
       <c r="Q25" s="24" t="s">
         <v>73</v>
@@ -2588,10 +2601,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I10</f>
         <v>24500</v>
       </c>
-      <c r="O26" s="26"/>
+      <c r="O26" s="26" t="n">
+        <v>38000</v>
+      </c>
       <c r="P26" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N26),ISNUMBER(O26)),N26*O26,0)</f>
-        <v>0</v>
+        <v>931000000</v>
       </c>
       <c r="Q26" s="24" t="s">
         <v>73</v>
@@ -2683,10 +2698,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I11</f>
         <v>3500</v>
       </c>
-      <c r="O28" s="26"/>
+      <c r="O28" s="26" t="n">
+        <v>37500</v>
+      </c>
       <c r="P28" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N28),ISNUMBER(O28)),N28*O28,0)</f>
-        <v>0</v>
+        <v>131250000</v>
       </c>
       <c r="Q28" s="24" t="s">
         <v>73</v>
@@ -2740,10 +2757,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I12</f>
         <v>7000</v>
       </c>
-      <c r="O29" s="26"/>
+      <c r="O29" s="26" t="n">
+        <v>35000</v>
+      </c>
       <c r="P29" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N29),ISNUMBER(O29)),N29*O29,0)</f>
-        <v>0</v>
+        <v>245000000</v>
       </c>
       <c r="Q29" s="24" t="s">
         <v>73</v>
@@ -2797,10 +2816,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I13</f>
         <v>10500</v>
       </c>
-      <c r="O30" s="26"/>
+      <c r="O30" s="26" t="n">
+        <v>42000</v>
+      </c>
       <c r="P30" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N30),ISNUMBER(O30)),N30*O30,0)</f>
-        <v>0</v>
+        <v>441000000</v>
       </c>
       <c r="Q30" s="24" t="s">
         <v>73</v>
@@ -2885,10 +2906,12 @@
         <f aca="false">J32</f>
         <v>6</v>
       </c>
-      <c r="O32" s="26"/>
+      <c r="O32" s="26" t="n">
+        <v>300000</v>
+      </c>
       <c r="P32" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N32),ISNUMBER(O32)),N32*O32,0)</f>
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="Q32" s="24" t="s">
         <v>139</v>
@@ -2933,10 +2956,12 @@
         <f aca="false">J33</f>
         <v>6</v>
       </c>
-      <c r="O33" s="26"/>
+      <c r="O33" s="26" t="n">
+        <v>300000</v>
+      </c>
       <c r="P33" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N33),ISNUMBER(O33)),N33*O33,0)</f>
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="Q33" s="24" t="s">
         <v>139</v>
@@ -2981,10 +3006,12 @@
         <f aca="false">J34</f>
         <v>6</v>
       </c>
-      <c r="O34" s="26"/>
+      <c r="O34" s="26" t="n">
+        <v>300000</v>
+      </c>
       <c r="P34" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N34),ISNUMBER(O34)),N34*O34,0)</f>
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="Q34" s="24" t="s">
         <v>139</v>
@@ -3029,10 +3056,12 @@
         <f aca="false">J35</f>
         <v>6</v>
       </c>
-      <c r="O35" s="26"/>
+      <c r="O35" s="26" t="n">
+        <v>300000</v>
+      </c>
       <c r="P35" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N35),ISNUMBER(O35)),N35*O35,0)</f>
-        <v>0</v>
+        <v>1800000</v>
       </c>
       <c r="Q35" s="24" t="s">
         <v>139</v>
@@ -3108,10 +3137,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I14</f>
         <v>13960</v>
       </c>
-      <c r="O37" s="26"/>
+      <c r="O37" s="26" t="n">
+        <v>38000</v>
+      </c>
       <c r="P37" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N37),ISNUMBER(O37)),N37*O37,0)</f>
-        <v>0</v>
+        <v>530480000</v>
       </c>
       <c r="Q37" s="24" t="s">
         <v>73</v>
@@ -3165,10 +3196,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I15</f>
         <v>860</v>
       </c>
-      <c r="O38" s="26"/>
+      <c r="O38" s="26" t="n">
+        <v>60000</v>
+      </c>
       <c r="P38" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N38),ISNUMBER(O38)),N38*O38,0)</f>
-        <v>0</v>
+        <v>51600000</v>
       </c>
       <c r="Q38" s="24" t="s">
         <v>73</v>
@@ -3262,10 +3295,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I16</f>
         <v>23220</v>
       </c>
-      <c r="O40" s="26"/>
+      <c r="O40" s="26" t="n">
+        <v>32000</v>
+      </c>
       <c r="P40" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N40),ISNUMBER(O40)),N40*O40,0)</f>
-        <v>0</v>
+        <v>743040000</v>
       </c>
       <c r="Q40" s="24" t="s">
         <v>73</v>
@@ -3317,10 +3352,12 @@
         <f aca="false">'4. Расчёт - Calculation'!I17</f>
         <v>3680</v>
       </c>
-      <c r="O41" s="26"/>
+      <c r="O41" s="26" t="n">
+        <v>32000</v>
+      </c>
       <c r="P41" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N41),ISNUMBER(O41)),N41*O41,0)</f>
-        <v>0</v>
+        <v>117760000</v>
       </c>
       <c r="Q41" s="24" t="s">
         <v>73</v>
@@ -3393,43 +3430,47 @@
         <f aca="false">J43</f>
         <v>1</v>
       </c>
-      <c r="O43" s="26"/>
+      <c r="O43" s="26" t="n">
+        <v>50000000</v>
+      </c>
       <c r="P43" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N43),ISNUMBER(O43)),N43*O43,0)</f>
-        <v>0</v>
+        <v>50000000</v>
       </c>
       <c r="Q43" s="24"/>
       <c r="R43" s="28"/>
       <c r="S43" s="28"/>
-      <c r="T43" s="24"/>
+      <c r="T43" s="24" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="22" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D44" s="23" t="s">
         <v>101</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F44" s="22" t="s">
         <v>59</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H44" s="23" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I44" s="22" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J44" s="29" t="n">
         <v>4</v>
@@ -3441,10 +3482,12 @@
         <f aca="false">J44</f>
         <v>4</v>
       </c>
-      <c r="O44" s="26"/>
+      <c r="O44" s="26" t="n">
+        <v>3200000</v>
+      </c>
       <c r="P44" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N44),ISNUMBER(O44)),N44*O44,0)</f>
-        <v>0</v>
+        <v>12800000</v>
       </c>
       <c r="Q44" s="24"/>
       <c r="R44" s="28"/>
@@ -3453,25 +3496,25 @@
     </row>
     <row r="45" customFormat="false" ht="107.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="22" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F45" s="22" t="s">
         <v>59</v>
       </c>
       <c r="G45" s="22" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H45" s="23"/>
       <c r="I45" s="22" t="s">
@@ -3487,41 +3530,45 @@
         <f aca="false">J45</f>
         <v>1</v>
       </c>
-      <c r="O45" s="26"/>
+      <c r="O45" s="26" t="n">
+        <v>60000000</v>
+      </c>
       <c r="P45" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N45),ISNUMBER(O45)),N45*O45,0)</f>
-        <v>0</v>
+        <v>60000000</v>
       </c>
       <c r="Q45" s="24"/>
       <c r="R45" s="28"/>
       <c r="S45" s="28"/>
-      <c r="T45" s="24"/>
+      <c r="T45" s="24" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F46" s="22" t="s">
         <v>59</v>
       </c>
       <c r="G46" s="22" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H46" s="23"/>
       <c r="I46" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J46" s="29" t="n">
         <v>1</v>
@@ -3533,10 +3580,12 @@
         <f aca="false">J46</f>
         <v>1</v>
       </c>
-      <c r="O46" s="26"/>
+      <c r="O46" s="26" t="n">
+        <v>5000000</v>
+      </c>
       <c r="P46" s="27" t="n">
         <f aca="false">IF(AND(ISNUMBER(N46),ISNUMBER(O46)),N46*O46,0)</f>
-        <v>0</v>
+        <v>5000000</v>
       </c>
       <c r="Q46" s="24"/>
       <c r="R46" s="28"/>
@@ -3545,7 +3594,7 @@
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="34" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B47" s="34"/>
       <c r="C47" s="34"/>
@@ -3563,7 +3612,7 @@
       <c r="O47" s="34"/>
       <c r="P47" s="35" t="n">
         <f aca="false">SUM(P18:P46)</f>
-        <v>361380000</v>
+        <v>5315430000</v>
       </c>
       <c r="Q47" s="36" t="str">
         <f aca="false">IF(K11="","",K11)</f>
@@ -3575,7 +3624,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="37" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B49" s="37"/>
       <c r="C49" s="37"/>
@@ -3591,7 +3640,7 @@
     </row>
     <row r="50" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="38" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B50" s="38"/>
       <c r="C50" s="38"/>
@@ -3607,7 +3656,7 @@
     </row>
     <row r="51" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="38" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B51" s="38"/>
       <c r="C51" s="38"/>
@@ -3623,7 +3672,7 @@
     </row>
     <row r="52" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="38" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B52" s="38"/>
       <c r="C52" s="38"/>
@@ -3639,7 +3688,7 @@
     </row>
     <row r="53" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="38" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B53" s="38"/>
       <c r="C53" s="38"/>
@@ -3726,17 +3775,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -3749,24 +3798,24 @@
         <v>32</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="39" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B6" s="39"/>
       <c r="C6" s="39"/>
@@ -3779,10 +3828,10 @@
         <v>1</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>110</v>
@@ -3797,10 +3846,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D8" s="22" t="s">
         <v>110</v>
@@ -3815,10 +3864,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>110</v>
@@ -3833,10 +3882,10 @@
         <v>4</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D10" s="22" t="s">
         <v>110</v>
@@ -3851,10 +3900,10 @@
         <v>5</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D11" s="22" t="s">
         <v>110</v>
@@ -3866,7 +3915,7 @@
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="39" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B12" s="39"/>
       <c r="C12" s="39"/>
@@ -3879,10 +3928,10 @@
         <v>6</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D13" s="22" t="s">
         <v>91</v>
@@ -3897,10 +3946,10 @@
         <v>7</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D14" s="22" t="s">
         <v>91</v>
@@ -3915,10 +3964,10 @@
         <v>8</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D15" s="22" t="s">
         <v>91</v>
@@ -3933,10 +3982,10 @@
         <v>9</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D16" s="22" t="s">
         <v>91</v>
@@ -3951,10 +4000,10 @@
         <v>10</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D17" s="22" t="s">
         <v>150</v>
@@ -3966,7 +4015,7 @@
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="39" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B18" s="39"/>
       <c r="C18" s="39"/>
@@ -3979,10 +4028,10 @@
         <v>11</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D19" s="22" t="s">
         <v>98</v>
@@ -3997,10 +4046,10 @@
         <v>12</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D20" s="22" t="s">
         <v>98</v>
@@ -4015,10 +4064,10 @@
         <v>13</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D21" s="22" t="s">
         <v>150</v>
@@ -4033,10 +4082,10 @@
         <v>14</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D22" s="22" t="s">
         <v>157</v>
@@ -4051,10 +4100,10 @@
         <v>15</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D23" s="22" t="s">
         <v>98</v>
@@ -4069,10 +4118,10 @@
         <v>16</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D24" s="22" t="s">
         <v>87</v>
@@ -4087,10 +4136,10 @@
         <v>17</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D25" s="22" t="s">
         <v>87</v>
@@ -4105,10 +4154,10 @@
         <v>18</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D26" s="22" t="s">
         <v>105</v>
@@ -4120,7 +4169,7 @@
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="39" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B27" s="39"/>
       <c r="C27" s="39"/>
@@ -4133,10 +4182,10 @@
         <v>19</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D28" s="22" t="s">
         <v>169</v>
@@ -4151,10 +4200,10 @@
         <v>20</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D29" s="22" t="s">
         <v>169</v>
@@ -4169,10 +4218,10 @@
         <v>21</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D30" s="22" t="s">
         <v>169</v>
@@ -4184,7 +4233,7 @@
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="39" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B31" s="39"/>
       <c r="C31" s="39"/>
@@ -4197,13 +4246,13 @@
         <v>22</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D32" s="22" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E32" s="40" t="s">
         <v>29</v>
@@ -4215,13 +4264,13 @@
         <v>23</v>
       </c>
       <c r="B33" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="C33" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="D33" s="22" t="s">
         <v>266</v>
-      </c>
-      <c r="C33" s="23" t="s">
-        <v>267</v>
-      </c>
-      <c r="D33" s="22" t="s">
-        <v>265</v>
       </c>
       <c r="E33" s="40" t="s">
         <v>29</v>
@@ -4230,7 +4279,7 @@
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="39" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B34" s="39"/>
       <c r="C34" s="39"/>
@@ -4243,10 +4292,10 @@
         <v>24</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D35" s="22" t="s">
         <v>173</v>
@@ -4261,10 +4310,10 @@
         <v>25</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D36" s="22" t="s">
         <v>173</v>
@@ -4279,10 +4328,10 @@
         <v>26</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D37" s="22" t="s">
         <v>173</v>
@@ -4297,10 +4346,10 @@
         <v>27</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D38" s="22" t="s">
         <v>173</v>
@@ -4315,13 +4364,13 @@
         <v>28</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D39" s="22" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E39" s="40" t="s">
         <v>29</v>
@@ -4333,13 +4382,13 @@
         <v>29</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D40" s="22" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E40" s="40" t="s">
         <v>29</v>
@@ -4348,7 +4397,7 @@
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="39" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B41" s="39"/>
       <c r="C41" s="39"/>
@@ -4361,13 +4410,13 @@
         <v>30</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E42" s="40" t="s">
         <v>29</v>
@@ -4376,7 +4425,7 @@
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="41" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B44" s="41"/>
       <c r="C44" s="41"/>
@@ -4433,44 +4482,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="42" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="43" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="44" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D4" s="44" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F4" s="44" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G4" s="44" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="H4" s="44" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="I4" s="44" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="J4" s="44" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4484,7 +4533,7 @@
         <v>452600</v>
       </c>
       <c r="D5" s="45" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E5" s="47" t="n">
         <v>3</v>
@@ -4493,7 +4542,7 @@
         <v>7</v>
       </c>
       <c r="G5" s="45" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H5" s="49" t="n">
         <f aca="false">C5*E5*F5/1000</f>
@@ -4504,7 +4553,7 @@
         <v>9510</v>
       </c>
       <c r="J5" s="45" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4518,7 +4567,7 @@
         <v>20</v>
       </c>
       <c r="D6" s="45" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E6" s="47" t="n">
         <v>30000</v>
@@ -4527,7 +4576,7 @@
         <v>3</v>
       </c>
       <c r="G6" s="45" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H6" s="49" t="n">
         <f aca="false">C6*E6*F6/1000</f>
@@ -4538,7 +4587,7 @@
         <v>1800</v>
       </c>
       <c r="J6" s="45" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4552,7 +4601,7 @@
         <v>20</v>
       </c>
       <c r="D7" s="45" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E7" s="47" t="n">
         <v>30000</v>
@@ -4561,7 +4610,7 @@
         <v>3</v>
       </c>
       <c r="G7" s="45" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H7" s="49" t="n">
         <f aca="false">C7*E7*F7/1000</f>
@@ -4572,7 +4621,7 @@
         <v>1800</v>
       </c>
       <c r="J7" s="45" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4586,7 +4635,7 @@
         <v>9200</v>
       </c>
       <c r="D8" s="45" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E8" s="47" t="n">
         <v>50</v>
@@ -4595,7 +4644,7 @@
         <v>14</v>
       </c>
       <c r="G8" s="45" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H8" s="49" t="n">
         <f aca="false">C8*E8*F8/1000</f>
@@ -4606,7 +4655,7 @@
         <v>6440</v>
       </c>
       <c r="J8" s="45" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4620,7 +4669,7 @@
         <v>102200</v>
       </c>
       <c r="D9" s="45" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E9" s="47" t="n">
         <v>25</v>
@@ -4629,7 +4678,7 @@
         <v>9</v>
       </c>
       <c r="G9" s="45" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="H9" s="49" t="n">
         <f aca="false">C9*E9*F9/1000</f>
@@ -4640,7 +4689,7 @@
         <v>23000</v>
       </c>
       <c r="J9" s="45" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4654,7 +4703,7 @@
         <v>35000</v>
       </c>
       <c r="D10" s="45" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E10" s="47" t="n">
         <v>50</v>
@@ -4663,7 +4712,7 @@
         <v>14</v>
       </c>
       <c r="G10" s="45" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H10" s="49" t="n">
         <f aca="false">C10*E10*F10/1000</f>
@@ -4674,7 +4723,7 @@
         <v>24500</v>
       </c>
       <c r="J10" s="45" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4688,7 +4737,7 @@
         <v>35000</v>
       </c>
       <c r="D11" s="45" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E11" s="47" t="n">
         <v>100</v>
@@ -4697,7 +4746,7 @@
         <v>1</v>
       </c>
       <c r="G11" s="45" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="H11" s="49" t="n">
         <f aca="false">C11*E11*F11/1000</f>
@@ -4708,7 +4757,7 @@
         <v>3500</v>
       </c>
       <c r="J11" s="45" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4722,7 +4771,7 @@
         <v>35000</v>
       </c>
       <c r="D12" s="45" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E12" s="47" t="n">
         <v>200</v>
@@ -4731,7 +4780,7 @@
         <v>1</v>
       </c>
       <c r="G12" s="45" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="H12" s="49" t="n">
         <f aca="false">C12*E12*F12/1000</f>
@@ -4742,7 +4791,7 @@
         <v>7000</v>
       </c>
       <c r="J12" s="45" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4756,7 +4805,7 @@
         <v>35000</v>
       </c>
       <c r="D13" s="45" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E13" s="47" t="n">
         <v>300</v>
@@ -4765,7 +4814,7 @@
         <v>1</v>
       </c>
       <c r="G13" s="45" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="H13" s="49" t="n">
         <f aca="false">C13*E13*F13/1000</f>
@@ -4776,7 +4825,7 @@
         <v>10500</v>
       </c>
       <c r="J13" s="45" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4790,7 +4839,7 @@
         <v>357700</v>
       </c>
       <c r="D14" s="45" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E14" s="47" t="n">
         <v>3</v>
@@ -4799,7 +4848,7 @@
         <v>13</v>
       </c>
       <c r="G14" s="45" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="H14" s="49" t="n">
         <f aca="false">C14*E14*F14/1000</f>
@@ -4810,7 +4859,7 @@
         <v>13960</v>
       </c>
       <c r="J14" s="45" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4824,7 +4873,7 @@
         <v>357700</v>
       </c>
       <c r="D15" s="45" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E15" s="47" t="n">
         <v>0.3</v>
@@ -4833,7 +4882,7 @@
         <v>8</v>
       </c>
       <c r="G15" s="45" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H15" s="49" t="n">
         <f aca="false">C15*E15*F15/1000</f>
@@ -4858,7 +4907,7 @@
         <v>193450</v>
       </c>
       <c r="D16" s="45" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E16" s="47" t="n">
         <v>15</v>
@@ -4867,7 +4916,7 @@
         <v>8</v>
       </c>
       <c r="G16" s="45" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H16" s="49" t="n">
         <f aca="false">C16*E16*F16/1000</f>
@@ -4878,7 +4927,7 @@
         <v>23220</v>
       </c>
       <c r="J16" s="45" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4892,7 +4941,7 @@
         <v>153300</v>
       </c>
       <c r="D17" s="45" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E17" s="47" t="n">
         <v>3</v>
@@ -4901,7 +4950,7 @@
         <v>8</v>
       </c>
       <c r="G17" s="45" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H17" s="49" t="n">
         <f aca="false">C17*E17*F17/1000</f>
@@ -4912,7 +4961,7 @@
         <v>3680</v>
       </c>
       <c r="J17" s="45" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
   </sheetData>

</xml_diff>